<commit_message>
Add morphometric features to trait model training and create labels.csv
- Updated `extract_features_from_images` function to include morphometric features: body length, withers height, heart girth, and hip length.
- Introduced a new `labels.csv` file containing image names, weights, morphometric measurements, and body condition scores for model training.
</commit_message>
<xml_diff>
--- a/measurements.xlsx
+++ b/measurements.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20398"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\g\Desktop\Data in brief\Cattle side and back view images\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aarya\OneDrive\Desktop\College stuff\VIT\TY\S6\EDI\Phenotyping\livestock-phenotyping-mvp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{648541A0-FA07-4E39-916D-DD644461E546}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{803D3E17-5BE7-490F-8C54-260925697786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="300" yWindow="495" windowWidth="28245" windowHeight="16095" xr2:uid="{24930DB0-56E5-EF4C-B7F1-753105A8A22A}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{24930DB0-56E5-EF4C-B7F1-753105A8A22A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Num</t>
   </si>
@@ -44,23 +44,26 @@
   <si>
     <t>Body weight (kg)</t>
   </si>
+  <si>
+    <t>BCS</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -68,7 +71,7 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -95,22 +98,16 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -126,7 +123,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -422,1494 +419,2071 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{227EFFE4-732B-E04E-BB91-D8398010239F}">
-  <dimension ref="A1:L74"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H73"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="11" style="1"/>
-    <col min="2" max="2" width="26.125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16.375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="26.09765625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="17.3984375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.3984375" style="1" customWidth="1"/>
     <col min="5" max="5" width="16.5" style="1" customWidth="1"/>
-    <col min="6" max="6" width="20.875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="20.8984375" style="1" customWidth="1"/>
     <col min="7" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:8">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="2" t="s">
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>161</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="1">
         <v>124</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="1">
         <v>190</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>47</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="1">
         <v>545</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+      <c r="G2" s="1">
+        <f>IF((F2/(B2*D2))*(E2/B2)&lt;0.004,2,
+IF((F2/(B2*D2))*(E2/B2)&lt;0.0045,2.5,
+IF((F2/(B2*D2))*(E2/B2)&lt;0.005,3,
+IF((F2/(B2*D2))*(E2/B2)&lt;0.0055,3.5,
+IF((F2/(B2*D2))*(E2/B2)&lt;0.006,4,4.5)))))</f>
+        <v>3.5</v>
+      </c>
+      <c r="H2" s="1">
+        <f>(F2/(B2*D2))*(E2/B2)</f>
+        <v>5.2010257888848504E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <v>152</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="1">
         <v>120</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="1">
         <v>183</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>43</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="1">
         <v>507</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2">
+      <c r="G3" s="1">
+        <f t="shared" ref="G3:G66" si="0">IF((F3/(B3*D3))*(E3/B3)&lt;0.004,2,
+IF((F3/(B3*D3))*(E3/B3)&lt;0.0045,2.5,
+IF((F3/(B3*D3))*(E3/B3)&lt;0.005,3,
+IF((F3/(B3*D3))*(E3/B3)&lt;0.0055,3.5,
+IF((F3/(B3*D3))*(E3/B3)&lt;0.006,4,4.5)))))</f>
+        <v>3.5</v>
+      </c>
+      <c r="H3" s="1">
+        <f t="shared" ref="H3:H66" si="1">(F3/(B3*D3))*(E3/B3)</f>
+        <v>5.1562996684982512E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1">
         <v>151</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="1">
         <v>124</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>179</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>41</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="1">
         <v>450</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+      <c r="G4" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H4" s="1">
+        <f t="shared" si="1"/>
+        <v>4.5205309283945453E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <v>174</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="1">
         <v>129</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="1">
         <v>202</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>50</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="1">
         <v>604</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+      <c r="G5" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H5" s="1">
+        <f t="shared" si="1"/>
+        <v>4.93806812310244E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="1">
         <v>128</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="1">
         <v>114</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="1">
         <v>176</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>41</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="1">
         <v>448</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+      <c r="G6" s="1">
+        <f t="shared" si="0"/>
+        <v>4.5</v>
+      </c>
+      <c r="H6" s="1">
+        <f t="shared" si="1"/>
+        <v>6.369850852272727E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="1">
         <v>138</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="1">
         <v>120</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="1">
         <v>180</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>42</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="1">
         <v>450</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+      <c r="G7" s="1">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H7" s="1">
+        <f t="shared" si="1"/>
+        <v>5.5135475740390677E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="1">
         <v>162</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="1">
         <v>124</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>182</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="1">
         <v>495</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
+      <c r="G8" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H8" s="1">
+        <f t="shared" si="1"/>
+        <v>4.6635463302129969E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="1">
         <v>154</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="1">
         <v>119</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="1">
         <v>174</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>41</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="1">
         <v>434</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+      <c r="G9" s="1">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+      <c r="H9" s="1">
+        <f t="shared" si="1"/>
+        <v>4.3120411458969447E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="1">
         <v>9</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="1">
         <v>142</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="1">
         <v>115</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="1">
         <v>170</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>42</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="1">
         <v>400</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
+      <c r="G10" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H10" s="1">
+        <f t="shared" si="1"/>
+        <v>4.900988365987141E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="1">
         <v>10</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="1">
         <v>156</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="1">
         <v>118</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="1">
         <v>180</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>44</v>
       </c>
-      <c r="F11" s="2">
+      <c r="F11" s="1">
         <v>467</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
+      <c r="G11" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H11" s="1">
+        <f t="shared" si="1"/>
+        <v>4.6908101395280889E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="1">
         <v>11</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="1">
         <v>145</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="1">
         <v>118</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>190</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>44</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F12" s="1">
         <v>466</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
+      <c r="G12" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H12" s="1">
+        <f t="shared" si="1"/>
+        <v>5.1327367169409855E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="1">
         <v>12</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" s="1">
         <v>138</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="1">
         <v>112</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>173</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>42</v>
       </c>
-      <c r="F13" s="2">
+      <c r="F13" s="1">
         <v>362</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
+      <c r="G13" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H13" s="1">
+        <f t="shared" si="1"/>
+        <v>4.6148074492535088E-3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="1">
         <v>13</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14" s="1">
         <v>151</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="1">
         <v>122</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>189</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46</v>
       </c>
-      <c r="F14" s="2">
+      <c r="F14" s="1">
         <v>444</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
+      <c r="G14" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H14" s="1">
+        <f t="shared" si="1"/>
+        <v>4.7394189756366856E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="1">
         <v>14</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15" s="1">
         <v>152</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="1">
         <v>121</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>181</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46</v>
       </c>
-      <c r="F15" s="2">
+      <c r="F15" s="1">
         <v>441</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
+      <c r="G15" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H15" s="1">
+        <f t="shared" si="1"/>
+        <v>4.8509932507919988E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="1">
         <v>15</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="1">
         <v>157</v>
       </c>
-      <c r="C16" s="2">
+      <c r="C16" s="1">
         <v>121</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>193</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>50</v>
       </c>
-      <c r="F16" s="2">
+      <c r="F16" s="1">
         <v>497</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
+      <c r="G16" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H16" s="1">
+        <f t="shared" si="1"/>
+        <v>5.2235983887353576E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" s="1">
         <v>16</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="1">
         <v>127</v>
       </c>
-      <c r="C17" s="2">
+      <c r="C17" s="1">
         <v>116</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>171</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>37</v>
       </c>
-      <c r="F17" s="2">
+      <c r="F17" s="1">
         <v>409</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
+      <c r="G17" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H17" s="1">
+        <f t="shared" si="1"/>
+        <v>5.4868296871096664E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" s="1">
         <v>17</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" s="1">
         <v>138</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C18" s="1">
         <v>117</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>168</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>41</v>
       </c>
-      <c r="F18" s="2">
+      <c r="F18" s="1">
         <v>371</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
+      <c r="G18" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H18" s="1">
+        <f t="shared" si="1"/>
+        <v>4.754340824756704E-3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="1">
         <v>18</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" s="1">
         <v>153</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19" s="1">
         <v>119</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>176</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>41</v>
       </c>
-      <c r="F19" s="2">
+      <c r="F19" s="1">
         <v>434</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
+      <c r="G19" s="1">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+      <c r="H19" s="1">
+        <f t="shared" si="1"/>
+        <v>4.3189488114516944E-3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="1">
         <v>19</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20" s="1">
         <v>138</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20" s="1">
         <v>115</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>173</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>44</v>
       </c>
-      <c r="F20" s="2">
+      <c r="F20" s="1">
         <v>367</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
+      <c r="G20" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H20" s="1">
+        <f t="shared" si="1"/>
+        <v>4.901335878094294E-3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" s="1">
         <v>20</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" s="1">
         <v>138</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C21" s="1">
         <v>112</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>173</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>42</v>
       </c>
-      <c r="F21" s="2">
+      <c r="F21" s="1">
         <v>362</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="2">
+      <c r="G21" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H21" s="1">
+        <f t="shared" si="1"/>
+        <v>4.6148074492535088E-3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" s="1">
         <v>21</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="1">
         <v>142</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C22" s="1">
         <v>118</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>174</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>43</v>
       </c>
-      <c r="F22" s="2">
+      <c r="F22" s="1">
         <v>403</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="2">
+      <c r="G22" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H22" s="1">
+        <f t="shared" si="1"/>
+        <v>4.9390971048893324E-3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" s="1">
         <v>22</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23" s="1">
         <v>142</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C23" s="1">
         <v>120</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>175</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45</v>
       </c>
-      <c r="F23" s="2">
+      <c r="F23" s="1">
         <v>440</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="2">
+      <c r="G23" s="1">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H23" s="1">
+        <f t="shared" si="1"/>
+        <v>5.6111315782016039E-3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" s="1">
         <v>23</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B24" s="1">
         <v>138</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C24" s="1">
         <v>112</v>
       </c>
-      <c r="D24" s="2">
+      <c r="D24" s="1">
         <v>173</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>44</v>
       </c>
-      <c r="F24" s="2">
+      <c r="F24" s="1">
         <v>362</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="2">
+      <c r="G24" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H24" s="1">
+        <f t="shared" si="1"/>
+        <v>4.8345601849322465E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" s="1">
         <v>24</v>
       </c>
-      <c r="B25" s="2">
+      <c r="B25" s="1">
         <v>144</v>
       </c>
-      <c r="C25" s="2">
+      <c r="C25" s="1">
         <v>122</v>
       </c>
-      <c r="D25" s="2">
+      <c r="D25" s="1">
         <v>186</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>44</v>
       </c>
-      <c r="F25" s="2">
+      <c r="F25" s="1">
         <v>445</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="2">
+      <c r="G25" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H25" s="1">
+        <f t="shared" si="1"/>
+        <v>5.0766212000530999E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" s="1">
         <v>25</v>
       </c>
-      <c r="B26" s="2">
+      <c r="B26" s="1">
         <v>138</v>
       </c>
-      <c r="C26" s="2">
+      <c r="C26" s="1">
         <v>112</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>173</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>44</v>
       </c>
-      <c r="F26" s="2">
+      <c r="F26" s="1">
         <v>362</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="2">
+      <c r="G26" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H26" s="1">
+        <f t="shared" si="1"/>
+        <v>4.8345601849322465E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" s="1">
         <v>26</v>
       </c>
-      <c r="B27" s="2">
+      <c r="B27" s="1">
         <v>156</v>
       </c>
-      <c r="C27" s="2">
+      <c r="C27" s="1">
         <v>118</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>180</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>44</v>
       </c>
-      <c r="F27" s="2">
+      <c r="F27" s="1">
         <v>467</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="2">
+      <c r="G27" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H27" s="1">
+        <f t="shared" si="1"/>
+        <v>4.6908101395280889E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
+      <c r="A28" s="1">
         <v>27</v>
       </c>
-      <c r="B28" s="2">
+      <c r="B28" s="1">
         <v>138</v>
       </c>
-      <c r="C28" s="2">
+      <c r="C28" s="1">
         <v>123</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>180</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>42</v>
       </c>
-      <c r="F28" s="2">
+      <c r="F28" s="1">
         <v>450</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="2">
+      <c r="G28" s="1">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H28" s="1">
+        <f t="shared" si="1"/>
+        <v>5.5135475740390677E-3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
+      <c r="A29" s="1">
         <v>28</v>
       </c>
-      <c r="B29" s="2">
+      <c r="B29" s="1">
         <v>167</v>
       </c>
-      <c r="C29" s="2">
+      <c r="C29" s="1">
         <v>128</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>192</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>29</v>
       </c>
-      <c r="F29" s="2">
+      <c r="F29" s="1">
         <v>601</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="2">
+      <c r="G29" s="1">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="H29" s="1">
+        <f t="shared" si="1"/>
+        <v>3.2549048609368091E-3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
+      <c r="A30" s="1">
         <v>29</v>
       </c>
-      <c r="B30" s="2">
+      <c r="B30" s="1">
         <v>154</v>
       </c>
-      <c r="C30" s="2">
+      <c r="C30" s="1">
         <v>118</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>194</v>
       </c>
-      <c r="E30" s="2">
+      <c r="E30" s="1">
         <v>45</v>
       </c>
-      <c r="F30" s="2">
+      <c r="F30" s="1">
         <v>550</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="2">
+      <c r="G30" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H30" s="1">
+        <f t="shared" si="1"/>
+        <v>5.3793776179637742E-3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
+      <c r="A31" s="1">
         <v>30</v>
       </c>
-      <c r="B31" s="2">
+      <c r="B31" s="1">
         <v>170</v>
       </c>
-      <c r="C31" s="2">
+      <c r="C31" s="1">
         <v>131</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>197</v>
       </c>
-      <c r="E31" s="2">
+      <c r="E31" s="1">
         <v>50</v>
       </c>
-      <c r="F31" s="2">
+      <c r="F31" s="1">
         <v>608</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="2">
+      <c r="G31" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H31" s="1">
+        <f t="shared" si="1"/>
+        <v>5.3396097166845237E-3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32" s="1">
         <v>31</v>
       </c>
-      <c r="B32" s="2">
+      <c r="B32" s="1">
         <v>155</v>
       </c>
-      <c r="C32" s="2">
+      <c r="C32" s="1">
         <v>120</v>
       </c>
-      <c r="D32" s="2">
+      <c r="D32" s="1">
         <v>186</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>44</v>
       </c>
-      <c r="F32" s="2">
+      <c r="F32" s="1">
         <v>486</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="2">
+      <c r="G32" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H32" s="1">
+        <f t="shared" si="1"/>
+        <v>4.7853378537142093E-3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33" s="1">
         <v>32</v>
       </c>
-      <c r="B33" s="2">
+      <c r="B33" s="1">
         <v>159</v>
       </c>
-      <c r="C33" s="2">
+      <c r="C33" s="1">
         <v>125</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>183</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>48</v>
       </c>
-      <c r="F33" s="2">
+      <c r="F33" s="1">
         <v>465</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="2">
+      <c r="G33" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H33" s="1">
+        <f t="shared" si="1"/>
+        <v>4.8244615764706338E-3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34" s="1">
         <v>33</v>
       </c>
-      <c r="B34" s="2">
+      <c r="B34" s="1">
         <v>138</v>
       </c>
-      <c r="C34" s="2">
+      <c r="C34" s="1">
         <v>123</v>
       </c>
-      <c r="D34" s="2">
+      <c r="D34" s="1">
         <v>180</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>42</v>
       </c>
-      <c r="F34" s="2">
+      <c r="F34" s="1">
         <v>450</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="2">
+      <c r="G34" s="1">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H34" s="1">
+        <f t="shared" si="1"/>
+        <v>5.5135475740390677E-3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35" s="1">
         <v>34</v>
       </c>
-      <c r="B35" s="2">
+      <c r="B35" s="1">
         <v>157</v>
       </c>
-      <c r="C35" s="2">
+      <c r="C35" s="1">
         <v>121</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>193</v>
       </c>
-      <c r="E35" s="2">
+      <c r="E35" s="1">
         <v>50</v>
       </c>
-      <c r="F35" s="2">
+      <c r="F35" s="1">
         <v>497</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="2">
+      <c r="G35" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H35" s="1">
+        <f t="shared" si="1"/>
+        <v>5.2235983887353576E-3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" s="1">
         <v>35</v>
       </c>
-      <c r="B36" s="2">
+      <c r="B36" s="1">
         <v>168</v>
       </c>
-      <c r="C36" s="2">
+      <c r="C36" s="1">
         <v>128</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>201</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>49</v>
       </c>
-      <c r="F36" s="2">
+      <c r="F36" s="1">
         <v>602</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="2">
+      <c r="G36" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H36" s="1">
+        <f t="shared" si="1"/>
+        <v>5.1996959646213375E-3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37" s="1">
         <v>36</v>
       </c>
-      <c r="B37" s="2">
+      <c r="B37" s="1">
         <v>142</v>
       </c>
-      <c r="C37" s="2">
+      <c r="C37" s="1">
         <v>118</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>174</v>
       </c>
-      <c r="E37" s="2">
+      <c r="E37" s="1">
         <v>43</v>
       </c>
-      <c r="F37" s="2">
+      <c r="F37" s="1">
         <v>400</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="2">
+      <c r="G37" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H37" s="1">
+        <f t="shared" si="1"/>
+        <v>4.9023296326444997E-3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" s="1">
         <v>37</v>
       </c>
-      <c r="B38" s="2">
+      <c r="B38" s="1">
         <v>170</v>
       </c>
-      <c r="C38" s="2">
+      <c r="C38" s="1">
         <v>130</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="1">
         <v>209</v>
       </c>
-      <c r="E38" s="2">
+      <c r="E38" s="1">
         <v>51</v>
       </c>
-      <c r="F38" s="2">
+      <c r="F38" s="1">
         <v>612</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="2">
+      <c r="G38" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H38" s="1">
+        <f t="shared" si="1"/>
+        <v>5.1674641148325351E-3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" s="1">
         <v>38</v>
       </c>
-      <c r="B39" s="2">
+      <c r="B39" s="1">
         <v>161</v>
       </c>
-      <c r="C39" s="2">
+      <c r="C39" s="1">
         <v>125</v>
       </c>
-      <c r="D39" s="2">
+      <c r="D39" s="1">
         <v>193</v>
       </c>
-      <c r="E39" s="2">
+      <c r="E39" s="1">
         <v>49</v>
       </c>
-      <c r="F39" s="2">
+      <c r="F39" s="1">
         <v>559</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="2">
+      <c r="G39" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H39" s="1">
+        <f t="shared" si="1"/>
+        <v>5.4751853629391662E-3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" s="1">
         <v>39</v>
       </c>
-      <c r="B40" s="2">
+      <c r="B40" s="1">
         <v>171</v>
       </c>
-      <c r="C40" s="2">
+      <c r="C40" s="1">
         <v>128</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="1">
         <v>204</v>
       </c>
-      <c r="E40" s="2">
+      <c r="E40" s="1">
         <v>50</v>
       </c>
-      <c r="F40" s="2">
+      <c r="F40" s="1">
         <v>617</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="2">
+      <c r="G40" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H40" s="1">
+        <f t="shared" si="1"/>
+        <v>5.17169351923937E-3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" s="1">
         <v>40</v>
       </c>
-      <c r="B41" s="2">
+      <c r="B41" s="1">
         <v>146</v>
       </c>
-      <c r="C41" s="2">
+      <c r="C41" s="1">
         <v>100</v>
       </c>
-      <c r="D41" s="2">
+      <c r="D41" s="1">
         <v>167</v>
       </c>
-      <c r="E41" s="2">
+      <c r="E41" s="1">
         <v>41</v>
       </c>
-      <c r="F41" s="2">
+      <c r="F41" s="1">
         <v>342</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="2">
+      <c r="G41" s="1">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="H41" s="1">
+        <f t="shared" si="1"/>
+        <v>3.939016319022679E-3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42" s="1">
         <v>41</v>
       </c>
-      <c r="B42" s="2">
+      <c r="B42" s="1">
         <v>145</v>
       </c>
-      <c r="C42" s="2">
+      <c r="C42" s="1">
         <v>121</v>
       </c>
-      <c r="D42" s="2">
+      <c r="D42" s="1">
         <v>190</v>
       </c>
-      <c r="E42" s="2">
+      <c r="E42" s="1">
         <v>44</v>
       </c>
-      <c r="F42" s="2">
+      <c r="F42" s="1">
         <v>479</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="2">
+      <c r="G42" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H42" s="1">
+        <f t="shared" si="1"/>
+        <v>5.2759246511045752E-3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43" s="1">
         <v>42</v>
       </c>
-      <c r="B43" s="2">
+      <c r="B43" s="1">
         <v>144</v>
       </c>
-      <c r="C43" s="2">
+      <c r="C43" s="1">
         <v>122</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="1">
         <v>186</v>
       </c>
-      <c r="E43" s="2">
+      <c r="E43" s="1">
         <v>44</v>
       </c>
-      <c r="F43" s="2">
+      <c r="F43" s="1">
         <v>445</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="2">
+      <c r="G43" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H43" s="1">
+        <f t="shared" si="1"/>
+        <v>5.0766212000530999E-3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44" s="1">
         <v>43</v>
       </c>
-      <c r="B44" s="2">
+      <c r="B44" s="1">
         <v>167</v>
       </c>
-      <c r="C44" s="2">
+      <c r="C44" s="1">
         <v>128</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="1">
         <v>192</v>
       </c>
-      <c r="E44" s="2">
+      <c r="E44" s="1">
         <v>29</v>
       </c>
-      <c r="F44" s="2">
+      <c r="F44" s="1">
         <v>601</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="2">
+      <c r="G44" s="1">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="H44" s="1">
+        <f t="shared" si="1"/>
+        <v>3.2549048609368091E-3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45" s="1">
         <v>44</v>
       </c>
-      <c r="B45" s="2">
+      <c r="B45" s="1">
         <v>161</v>
       </c>
-      <c r="C45" s="2">
+      <c r="C45" s="1">
         <v>125</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>193</v>
       </c>
-      <c r="E45" s="2">
+      <c r="E45" s="1">
         <v>49</v>
       </c>
-      <c r="F45" s="2">
+      <c r="F45" s="1">
         <v>565</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="2">
+      <c r="G45" s="1">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H45" s="1">
+        <f t="shared" si="1"/>
+        <v>5.5339530054751857E-3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="A46" s="1">
         <v>45</v>
       </c>
-      <c r="B46" s="2">
+      <c r="B46" s="1">
         <v>146</v>
       </c>
-      <c r="C46" s="2">
+      <c r="C46" s="1">
         <v>100</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>167</v>
       </c>
-      <c r="E46" s="2">
+      <c r="E46" s="1">
         <v>41</v>
       </c>
-      <c r="F46" s="2">
+      <c r="F46" s="1">
         <v>341</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="2">
+      <c r="G46" s="1">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="H46" s="1">
+        <f t="shared" si="1"/>
+        <v>3.9274987274465897E-3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="A47" s="1">
         <v>46</v>
       </c>
-      <c r="B47" s="2">
+      <c r="B47" s="1">
         <v>148</v>
       </c>
-      <c r="C47" s="2">
+      <c r="C47" s="1">
         <v>100</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="1">
         <v>167</v>
       </c>
-      <c r="E47" s="2">
+      <c r="E47" s="1">
         <v>41</v>
       </c>
-      <c r="F47" s="2">
+      <c r="F47" s="1">
         <v>353</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="2">
+      <c r="G47" s="1">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="H47" s="1">
+        <f t="shared" si="1"/>
+        <v>3.9565682367915739E-3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
+      <c r="A48" s="1">
         <v>47</v>
       </c>
-      <c r="B48" s="2">
+      <c r="B48" s="1">
         <v>157</v>
       </c>
-      <c r="C48" s="2">
+      <c r="C48" s="1">
         <v>125</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="1">
         <v>192</v>
       </c>
-      <c r="E48" s="2">
+      <c r="E48" s="1">
         <v>51</v>
       </c>
-      <c r="F48" s="2">
+      <c r="F48" s="1">
         <v>511</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="2">
+      <c r="G48" s="1">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H48" s="1">
+        <f t="shared" si="1"/>
+        <v>5.5066889123291003E-3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49" s="1">
         <v>48</v>
       </c>
-      <c r="B49" s="2">
+      <c r="B49" s="1">
         <v>155</v>
       </c>
-      <c r="C49" s="2">
+      <c r="C49" s="1">
         <v>120</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="1">
         <v>186</v>
       </c>
-      <c r="E49" s="2">
+      <c r="E49" s="1">
         <v>44</v>
       </c>
-      <c r="F49" s="2">
+      <c r="F49" s="1">
         <v>486</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="2">
+      <c r="G49" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H49" s="1">
+        <f t="shared" si="1"/>
+        <v>4.7853378537142093E-3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50" s="1">
         <v>49</v>
       </c>
-      <c r="B50" s="2">
+      <c r="B50" s="1">
         <v>146</v>
       </c>
-      <c r="C50" s="2">
+      <c r="C50" s="1">
         <v>100</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="1">
         <v>167</v>
       </c>
-      <c r="E50" s="2">
+      <c r="E50" s="1">
         <v>41</v>
       </c>
-      <c r="F50" s="2">
+      <c r="F50" s="1">
         <v>342</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="2">
+      <c r="G50" s="1">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="H50" s="1">
+        <f t="shared" si="1"/>
+        <v>3.939016319022679E-3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51" s="1">
         <v>50</v>
       </c>
-      <c r="B51" s="2">
+      <c r="B51" s="1">
         <v>167</v>
       </c>
-      <c r="C51" s="2">
+      <c r="C51" s="1">
         <v>130</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>190</v>
       </c>
-      <c r="E51" s="2">
+      <c r="E51" s="1">
         <v>50</v>
       </c>
-      <c r="F51" s="2">
+      <c r="F51" s="1">
         <v>600</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="2">
+      <c r="G51" s="1">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H51" s="1">
+        <f t="shared" si="1"/>
+        <v>5.6615417132957532E-3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
+      <c r="A52" s="1">
         <v>51</v>
       </c>
-      <c r="B52" s="2">
+      <c r="B52" s="1">
         <v>138</v>
       </c>
-      <c r="C52" s="2">
+      <c r="C52" s="1">
         <v>123</v>
       </c>
-      <c r="D52" s="2">
+      <c r="D52" s="1">
         <v>180</v>
       </c>
-      <c r="E52" s="2">
+      <c r="E52" s="1">
         <v>42</v>
       </c>
-      <c r="F52" s="2">
+      <c r="F52" s="1">
         <v>450</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" s="2">
+      <c r="G52" s="1">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H52" s="1">
+        <f t="shared" si="1"/>
+        <v>5.5135475740390677E-3</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
+      <c r="A53" s="1">
         <v>52</v>
       </c>
-      <c r="B53" s="2">
+      <c r="B53" s="1">
         <v>150</v>
       </c>
-      <c r="C53" s="2">
+      <c r="C53" s="1">
         <v>118</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>176</v>
       </c>
-      <c r="E53" s="2">
+      <c r="E53" s="1">
         <v>46</v>
       </c>
-      <c r="F53" s="2">
+      <c r="F53" s="1">
         <v>443</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" s="2">
+      <c r="G53" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H53" s="1">
+        <f t="shared" si="1"/>
+        <v>5.1459595959595953E-3</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
+      <c r="A54" s="1">
         <v>53</v>
       </c>
-      <c r="B54" s="2">
+      <c r="B54" s="1">
         <v>154</v>
       </c>
-      <c r="C54" s="2">
+      <c r="C54" s="1">
         <v>118</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>194</v>
       </c>
-      <c r="E54" s="2">
+      <c r="E54" s="1">
         <v>45</v>
       </c>
-      <c r="F54" s="2">
+      <c r="F54" s="1">
         <v>550</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="2">
+      <c r="G54" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H54" s="1">
+        <f t="shared" si="1"/>
+        <v>5.3793776179637742E-3</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
+      <c r="A55" s="1">
         <v>54</v>
       </c>
-      <c r="B55" s="2">
+      <c r="B55" s="1">
         <v>151</v>
       </c>
-      <c r="C55" s="2">
+      <c r="C55" s="1">
         <v>122</v>
       </c>
-      <c r="D55" s="2">
+      <c r="D55" s="1">
         <v>189</v>
       </c>
-      <c r="E55" s="2">
+      <c r="E55" s="1">
         <v>46</v>
       </c>
-      <c r="F55" s="2">
+      <c r="F55" s="1">
         <v>444</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" s="2">
+      <c r="G55" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H55" s="1">
+        <f t="shared" si="1"/>
+        <v>4.7394189756366856E-3</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
+      <c r="A56" s="1">
         <v>55</v>
       </c>
-      <c r="B56" s="2">
+      <c r="B56" s="1">
         <v>157</v>
       </c>
-      <c r="C56" s="2">
+      <c r="C56" s="1">
         <v>121</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>193</v>
       </c>
-      <c r="E56" s="2">
+      <c r="E56" s="1">
         <v>50</v>
       </c>
-      <c r="F56" s="2">
+      <c r="F56" s="1">
         <v>497</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="2">
+      <c r="G56" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H56" s="1">
+        <f t="shared" si="1"/>
+        <v>5.2235983887353576E-3</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
+      <c r="A57" s="1">
         <v>56</v>
       </c>
-      <c r="B57" s="2">
+      <c r="B57" s="1">
         <v>150</v>
       </c>
-      <c r="C57" s="2">
+      <c r="C57" s="1">
         <v>118</v>
       </c>
-      <c r="D57" s="2">
+      <c r="D57" s="1">
         <v>175</v>
       </c>
-      <c r="E57" s="2">
+      <c r="E57" s="1">
         <v>42</v>
       </c>
-      <c r="F57" s="2">
+      <c r="F57" s="1">
         <v>408</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" s="2">
+      <c r="G57" s="1">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+      <c r="H57" s="1">
+        <f t="shared" si="1"/>
+        <v>4.3520000000000008E-3</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
+      <c r="A58" s="1">
         <v>57</v>
       </c>
-      <c r="B58" s="2">
+      <c r="B58" s="1">
         <v>146</v>
       </c>
-      <c r="C58" s="2">
+      <c r="C58" s="1">
         <v>100</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58" s="1">
         <v>167</v>
       </c>
-      <c r="E58" s="2">
+      <c r="E58" s="1">
         <v>41</v>
       </c>
-      <c r="F58" s="2">
+      <c r="F58" s="1">
         <v>346</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="2">
+      <c r="G58" s="1">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="H58" s="1">
+        <f t="shared" si="1"/>
+        <v>3.9850866853270378E-3</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
+      <c r="A59" s="1">
         <v>58</v>
       </c>
-      <c r="B59" s="2">
+      <c r="B59" s="1">
         <v>159</v>
       </c>
-      <c r="C59" s="2">
+      <c r="C59" s="1">
         <v>125</v>
       </c>
-      <c r="D59" s="2">
+      <c r="D59" s="1">
         <v>183</v>
       </c>
-      <c r="E59" s="2">
+      <c r="E59" s="1">
         <v>48</v>
       </c>
-      <c r="F59" s="2">
+      <c r="F59" s="1">
         <v>465</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="2">
+      <c r="G59" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H59" s="1">
+        <f t="shared" si="1"/>
+        <v>4.8244615764706338E-3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
+      <c r="A60" s="1">
         <v>59</v>
       </c>
-      <c r="B60" s="2">
+      <c r="B60" s="1">
         <v>168</v>
       </c>
-      <c r="C60" s="2">
+      <c r="C60" s="1">
         <v>128</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>201</v>
       </c>
-      <c r="E60" s="2">
+      <c r="E60" s="1">
         <v>49</v>
       </c>
-      <c r="F60" s="2">
+      <c r="F60" s="1">
         <v>602</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="2">
+      <c r="G60" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H60" s="1">
+        <f t="shared" si="1"/>
+        <v>5.1996959646213375E-3</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8">
+      <c r="A61" s="1">
         <v>60</v>
       </c>
-      <c r="B61" s="2">
+      <c r="B61" s="1">
         <v>157</v>
       </c>
-      <c r="C61" s="2">
+      <c r="C61" s="1">
         <v>121</v>
       </c>
-      <c r="D61" s="2">
+      <c r="D61" s="1">
         <v>193</v>
       </c>
-      <c r="E61" s="2">
+      <c r="E61" s="1">
         <v>50</v>
       </c>
-      <c r="F61" s="2">
+      <c r="F61" s="1">
         <v>497</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="2">
+      <c r="G61" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H61" s="1">
+        <f t="shared" si="1"/>
+        <v>5.2235983887353576E-3</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
+      <c r="A62" s="1">
         <v>61</v>
       </c>
-      <c r="B62" s="2">
+      <c r="B62" s="1">
         <v>167</v>
       </c>
-      <c r="C62" s="2">
+      <c r="C62" s="1">
         <v>128</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62" s="1">
         <v>192</v>
       </c>
-      <c r="E62" s="2">
+      <c r="E62" s="1">
         <v>29</v>
       </c>
-      <c r="F62" s="2">
+      <c r="F62" s="1">
         <v>601</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="2">
+      <c r="G62" s="1">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="H62" s="1">
+        <f t="shared" si="1"/>
+        <v>3.2549048609368091E-3</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8">
+      <c r="A63" s="1">
         <v>62</v>
       </c>
-      <c r="B63" s="2">
+      <c r="B63" s="1">
         <v>161</v>
       </c>
-      <c r="C63" s="2">
+      <c r="C63" s="1">
         <v>125</v>
       </c>
-      <c r="D63" s="2">
+      <c r="D63" s="1">
         <v>193</v>
       </c>
-      <c r="E63" s="2">
+      <c r="E63" s="1">
         <v>49</v>
       </c>
-      <c r="F63" s="2">
+      <c r="F63" s="1">
         <v>586</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="2">
+      <c r="G63" s="1">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H63" s="1">
+        <f t="shared" si="1"/>
+        <v>5.7396397543512546E-3</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8">
+      <c r="A64" s="1">
         <v>63</v>
       </c>
-      <c r="B64" s="2">
+      <c r="B64" s="1">
         <v>170</v>
       </c>
-      <c r="C64" s="2">
+      <c r="C64" s="1">
         <v>131</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="1">
         <v>197</v>
       </c>
-      <c r="E64" s="2">
+      <c r="E64" s="1">
         <v>50</v>
       </c>
-      <c r="F64" s="2">
+      <c r="F64" s="1">
         <v>608</v>
       </c>
-    </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A65" s="2">
+      <c r="G64" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H64" s="1">
+        <f t="shared" si="1"/>
+        <v>5.3396097166845237E-3</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8">
+      <c r="A65" s="1">
         <v>64</v>
       </c>
-      <c r="B65" s="2">
+      <c r="B65" s="1">
         <v>173</v>
       </c>
-      <c r="C65" s="2">
+      <c r="C65" s="1">
         <v>130</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>200</v>
       </c>
-      <c r="E65" s="2">
+      <c r="E65" s="1">
         <v>48</v>
       </c>
-      <c r="F65" s="2">
+      <c r="F65" s="1">
         <v>610</v>
       </c>
-    </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A66" s="2">
+      <c r="G65" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H65" s="1">
+        <f t="shared" si="1"/>
+        <v>4.8915767315981153E-3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8">
+      <c r="A66" s="1">
         <v>65</v>
       </c>
-      <c r="B66" s="2">
+      <c r="B66" s="1">
         <v>144</v>
       </c>
-      <c r="C66" s="2">
+      <c r="C66" s="1">
         <v>122</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66" s="1">
         <v>186</v>
       </c>
-      <c r="E66" s="2">
+      <c r="E66" s="1">
         <v>44</v>
       </c>
-      <c r="F66" s="2">
+      <c r="F66" s="1">
         <v>445</v>
       </c>
-    </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A67" s="2">
+      <c r="G66" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="H66" s="1">
+        <f t="shared" si="1"/>
+        <v>5.0766212000530999E-3</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8">
+      <c r="A67" s="1">
         <v>66</v>
       </c>
-      <c r="B67" s="2">
+      <c r="B67" s="1">
         <v>146</v>
       </c>
-      <c r="C67" s="2">
+      <c r="C67" s="1">
         <v>100</v>
       </c>
-      <c r="D67" s="2">
+      <c r="D67" s="1">
         <v>167</v>
       </c>
-      <c r="E67" s="2">
+      <c r="E67" s="1">
         <v>41</v>
       </c>
-      <c r="F67" s="2">
+      <c r="F67" s="1">
         <v>346</v>
       </c>
-    </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A68" s="2">
+      <c r="G67" s="1">
+        <f t="shared" ref="G67:G73" si="2">IF((F67/(B67*D67))*(E67/B67)&lt;0.004,2,
+IF((F67/(B67*D67))*(E67/B67)&lt;0.0045,2.5,
+IF((F67/(B67*D67))*(E67/B67)&lt;0.005,3,
+IF((F67/(B67*D67))*(E67/B67)&lt;0.0055,3.5,
+IF((F67/(B67*D67))*(E67/B67)&lt;0.006,4,4.5)))))</f>
+        <v>2</v>
+      </c>
+      <c r="H67" s="1">
+        <f t="shared" ref="H67:H73" si="3">(F67/(B67*D67))*(E67/B67)</f>
+        <v>3.9850866853270378E-3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8">
+      <c r="A68" s="1">
         <v>67</v>
       </c>
-      <c r="B68" s="2">
+      <c r="B68" s="1">
         <v>155</v>
       </c>
-      <c r="C68" s="2">
+      <c r="C68" s="1">
         <v>120</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D68" s="1">
         <v>186</v>
       </c>
-      <c r="E68" s="2">
+      <c r="E68" s="1">
         <v>44</v>
       </c>
-      <c r="F68" s="2">
+      <c r="F68" s="1">
         <v>486</v>
       </c>
-    </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A69" s="2">
+      <c r="G68" s="1">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="H68" s="1">
+        <f t="shared" si="3"/>
+        <v>4.7853378537142093E-3</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8">
+      <c r="A69" s="1">
         <v>68</v>
       </c>
-      <c r="B69" s="2">
+      <c r="B69" s="1">
         <v>171</v>
       </c>
-      <c r="C69" s="2">
+      <c r="C69" s="1">
         <v>128</v>
       </c>
-      <c r="D69" s="2">
+      <c r="D69" s="1">
         <v>204</v>
       </c>
-      <c r="E69" s="2">
+      <c r="E69" s="1">
         <v>50</v>
       </c>
-      <c r="F69" s="2">
+      <c r="F69" s="1">
         <v>617</v>
       </c>
-    </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A70" s="2">
+      <c r="G69" s="1">
+        <f t="shared" si="2"/>
+        <v>3.5</v>
+      </c>
+      <c r="H69" s="1">
+        <f t="shared" si="3"/>
+        <v>5.17169351923937E-3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8">
+      <c r="A70" s="1">
         <v>69</v>
       </c>
-      <c r="B70" s="2">
+      <c r="B70" s="1">
         <v>155</v>
       </c>
-      <c r="C70" s="2">
+      <c r="C70" s="1">
         <v>120</v>
       </c>
-      <c r="D70" s="2">
+      <c r="D70" s="1">
         <v>183</v>
       </c>
-      <c r="E70" s="2">
+      <c r="E70" s="1">
         <v>44</v>
       </c>
-      <c r="F70" s="2">
+      <c r="F70" s="1">
         <v>512</v>
       </c>
-    </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A71" s="2">
+      <c r="G70" s="1">
+        <f t="shared" si="2"/>
+        <v>3.5</v>
+      </c>
+      <c r="H70" s="1">
+        <f t="shared" si="3"/>
+        <v>5.123988559276255E-3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8">
+      <c r="A71" s="1">
         <v>70</v>
       </c>
-      <c r="B71" s="2">
+      <c r="B71" s="1">
         <v>174</v>
       </c>
-      <c r="C71" s="2">
+      <c r="C71" s="1">
         <v>137</v>
       </c>
-      <c r="D71" s="2">
+      <c r="D71" s="1">
         <v>221</v>
       </c>
-      <c r="E71" s="2">
+      <c r="E71" s="1">
         <v>49</v>
       </c>
-      <c r="F71" s="2">
+      <c r="F71" s="1">
         <v>644</v>
       </c>
-    </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A72" s="2">
+      <c r="G71" s="1">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="H71" s="1">
+        <f t="shared" si="3"/>
+        <v>4.7161887408092911E-3</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8">
+      <c r="A72" s="1">
         <v>71</v>
       </c>
-      <c r="B72" s="2">
+      <c r="B72" s="1">
         <v>161</v>
       </c>
-      <c r="C72" s="2">
+      <c r="C72" s="1">
         <v>125</v>
       </c>
-      <c r="D72" s="2">
+      <c r="D72" s="1">
         <v>193</v>
       </c>
-      <c r="E72" s="2">
+      <c r="E72" s="1">
         <v>49</v>
       </c>
-      <c r="F72" s="2">
+      <c r="F72" s="1">
         <v>586</v>
       </c>
-    </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A73" s="2">
+      <c r="G72" s="1">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="H72" s="1">
+        <f t="shared" si="3"/>
+        <v>5.7396397543512546E-3</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8">
+      <c r="A73" s="1">
         <v>72</v>
       </c>
-      <c r="B73" s="2">
+      <c r="B73" s="1">
         <v>156</v>
       </c>
-      <c r="C73" s="2">
+      <c r="C73" s="1">
         <v>114</v>
       </c>
-      <c r="D73" s="2">
+      <c r="D73" s="1">
         <v>189</v>
       </c>
-      <c r="E73" s="2">
+      <c r="E73" s="1">
         <v>46</v>
       </c>
-      <c r="F73" s="2">
+      <c r="F73" s="1">
         <v>567</v>
       </c>
-    </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A74" s="2"/>
-      <c r="B74" s="2"/>
-      <c r="C74" s="2"/>
-      <c r="D74" s="2"/>
-      <c r="E74" s="2"/>
-      <c r="F74" s="2"/>
-      <c r="G74" s="2"/>
-      <c r="H74" s="3"/>
-      <c r="I74" s="3"/>
-      <c r="J74" s="3"/>
-      <c r="K74" s="3"/>
-      <c r="L74" s="2"/>
+      <c r="G73" s="1">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="H73" s="1">
+        <f t="shared" si="3"/>
+        <v>5.6706114398422094E-3</v>
+      </c>
     </row>
   </sheetData>
-  <sortState ref="A2:F70">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F70">
     <sortCondition ref="A1"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>